<commit_message>
docs(backlog): re-estimate lost venue recovery to five points
E10-S05 / SCRUM-74: reconcile the whole-story estimate with the four current scenarios; update both backlog views and regenerate CAA 261026 for teammate review.
</commit_message>
<xml_diff>
--- a/docs/CONNECTSPHERE BACKLOGS CAA 261026.xlsx
+++ b/docs/CONNECTSPHERE BACKLOGS CAA 261026.xlsx
@@ -3904,7 +3904,7 @@
       <c r="E62" s="2" t="inlineStr">
         <is>
           <t>As an Event Coordinator, I want to be alerted when a venue becomes unavailable for one of my events and to find and request a replacement from the event itself, so that I can arrange an alternative before Attendees are affected while the original event information is preserved.
-Returned to Release 1 by the Week 7 Customer Changes (C-66, T-67). The three-point estimate is carried from the original backlog and re-estimated at Sprint 3 planning (T-73). The alert itself is raised by E05-S06; this story is what the Coordinator does with it.
+Returned to Release 1 by the Week 7 Customer Changes (C-66, T-67). The original estimate was three points. Re-estimated to five points on 26 October 2026 at the story owner's request, with the change recorded for teammate review through the estimate PR. The four current scenarios include lost-booking context and same-event replacement search, linked replacement requests, explicit cancellation only after confirmation, and effective-change publication/notification timing with integration and rollback testing. This is the whole-story estimate, not remaining work or elapsed waiting time. E05-S06 still owns the unavailability trigger and Confirmed-to-Planning transition; that implementation is not counted again here.
 Updated on 23 October 2026, before any work on the story started, to the Week 9 decisions that closed O-24 and O-25; an incomplete story's criteria are updated in place (T-74). T-81 returns a Confirmed event that loses its venue to Planning without cancelling it (C-120), replacing the earlier "status unchanged" default in Scenario 1. C-121 confirms the Scenario 4 notification rule.</t>
         </is>
       </c>
@@ -3927,7 +3927,7 @@
         </is>
       </c>
       <c r="G62" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
@@ -7760,7 +7760,7 @@
       <c r="E72" s="2" t="inlineStr">
         <is>
           <t>As an Event Coordinator, I want to be alerted when a venue becomes unavailable for one of my events and to find and request a replacement from the event itself, so that I can arrange an alternative before Attendees are affected while the original event information is preserved.
-Returned to Release 1 by the Week 7 Customer Changes (C-66, T-67). The three-point estimate is carried from the original backlog and re-estimated at Sprint 3 planning (T-73). The alert itself is raised by E05-S06; this story is what the Coordinator does with it.
+Returned to Release 1 by the Week 7 Customer Changes (C-66, T-67). The original estimate was three points. Re-estimated to five points on 26 October 2026 at the story owner's request, with the change recorded for teammate review through the estimate PR. The four current scenarios include lost-booking context and same-event replacement search, linked replacement requests, explicit cancellation only after confirmation, and effective-change publication/notification timing with integration and rollback testing. This is the whole-story estimate, not remaining work or elapsed waiting time. E05-S06 still owns the unavailability trigger and Confirmed-to-Planning transition; that implementation is not counted again here.
 Updated on 23 October 2026, before any work on the story started, to the Week 9 decisions that closed O-24 and O-25; an incomplete story's criteria are updated in place (T-74). T-81 returns a Confirmed event that loses its venue to Planning without cancelling it (C-120), replacing the earlier "status unchanged" default in Scenario 1. C-121 confirms the Scenario 4 notification rule.</t>
         </is>
       </c>
@@ -7783,7 +7783,7 @@
         </is>
       </c>
       <c r="G72" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs(backlog): clarify estimate proposal and defer Jira reconciliation
Address Le Xin's review on #356. SCRUM-74 restored to 3 until the backlog proposal merges. Clarify T-73 and pending team confirmation; fix handoff spacing and append a readable correction without editing immutable evidence.
</commit_message>
<xml_diff>
--- a/docs/CONNECTSPHERE BACKLOGS CAA 261026.xlsx
+++ b/docs/CONNECTSPHERE BACKLOGS CAA 261026.xlsx
@@ -3904,7 +3904,7 @@
       <c r="E62" s="2" t="inlineStr">
         <is>
           <t>As an Event Coordinator, I want to be alerted when a venue becomes unavailable for one of my events and to find and request a replacement from the event itself, so that I can arrange an alternative before Attendees are affected while the original event information is preserved.
-Returned to Release 1 by the Week 7 Customer Changes (C-66, T-67). The original estimate was three points. Re-estimated to five points on 26 October 2026 at the story owner's request, with the change recorded for teammate review through the estimate PR. The four current scenarios include lost-booking context and same-event replacement search, linked replacement requests, explicit cancellation only after confirmation, and effective-change publication/notification timing with integration and rollback testing. This is the whole-story estimate, not remaining work or elapsed waiting time. E05-S06 still owns the unavailability trigger and Confirmed-to-Planning transition; that implementation is not counted again here.
+Returned to Release 1 by the Week 7 Customer Changes (C-66, T-67). The original estimate was three points. A five-point re-estimate was proposed on 26 October 2026 at the story owner's request for teammate review. Jira remains at three points until the matching backlog PR merges, then is reconciled to five points. The four current scenarios include lost-booking context and same-event replacement search, linked replacement requests, explicit cancellation only after confirmation, and effective-change publication/notification timing with integration and rollback testing. T-73 estimates in-flight stories for their remaining work only. Because the criteria changed on 23 October before implementation began, team/PO confirmation is required on whether five points records the revised pre-implementation size and how it is counted for sprint reporting. It is not an agreed estimate of work remaining now, and original commitments and historical estimates must be preserved. Elapsed waiting time is not story-point effort. E05-S06 still owns the unavailability trigger and Confirmed-to-Planning transition; that implementation is not counted again here.
 Updated on 23 October 2026, before any work on the story started, to the Week 9 decisions that closed O-24 and O-25; an incomplete story's criteria are updated in place (T-74). T-81 returns a Confirmed event that loses its venue to Planning without cancelling it (C-120), replacing the earlier "status unchanged" default in Scenario 1. C-121 confirms the Scenario 4 notification rule.</t>
         </is>
       </c>
@@ -7760,7 +7760,7 @@
       <c r="E72" s="2" t="inlineStr">
         <is>
           <t>As an Event Coordinator, I want to be alerted when a venue becomes unavailable for one of my events and to find and request a replacement from the event itself, so that I can arrange an alternative before Attendees are affected while the original event information is preserved.
-Returned to Release 1 by the Week 7 Customer Changes (C-66, T-67). The original estimate was three points. Re-estimated to five points on 26 October 2026 at the story owner's request, with the change recorded for teammate review through the estimate PR. The four current scenarios include lost-booking context and same-event replacement search, linked replacement requests, explicit cancellation only after confirmation, and effective-change publication/notification timing with integration and rollback testing. This is the whole-story estimate, not remaining work or elapsed waiting time. E05-S06 still owns the unavailability trigger and Confirmed-to-Planning transition; that implementation is not counted again here.
+Returned to Release 1 by the Week 7 Customer Changes (C-66, T-67). The original estimate was three points. A five-point re-estimate was proposed on 26 October 2026 at the story owner's request for teammate review. Jira remains at three points until the matching backlog PR merges, then is reconciled to five points. The four current scenarios include lost-booking context and same-event replacement search, linked replacement requests, explicit cancellation only after confirmation, and effective-change publication/notification timing with integration and rollback testing. T-73 estimates in-flight stories for their remaining work only. Because the criteria changed on 23 October before implementation began, team/PO confirmation is required on whether five points records the revised pre-implementation size and how it is counted for sprint reporting. It is not an agreed estimate of work remaining now, and original commitments and historical estimates must be preserved. Elapsed waiting time is not story-point effort. E05-S06 still owns the unavailability trigger and Confirmed-to-Planning transition; that implementation is not counted again here.
 Updated on 23 October 2026, before any work on the story started, to the Week 9 decisions that closed O-24 and O-25; an incomplete story's criteria are updated in place (T-74). T-81 returns a Confirmed event that loses its venue to Planning without cancelling it (C-120), replacing the earlier "status unchanged" default in Scenario 1. C-121 confirms the Scenario 4 notification rule.</t>
         </is>
       </c>

</xml_diff>